<commit_message>
Repair stale matiere_source labels after the england alias
Seven works still carried matiere_source = "override" from corrections
that the england -> Other alias made redundant and that were removed
from the sheets: the five Bueve de Hanstonne branches and Gui de Warwick
(French, storyverse-resolved) and Alpharts Tod (German, local). Their
provenance is restored, and an assertion now holds in both languages:
matiere_source == "override" exactly on the works the sheet overrides.

Final provenance: french 219 storyverse / 67 local / 27 override,
german 57 / 80 / 6. Analysis unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/french_works.xlsx
+++ b/data/french_works.xlsx
@@ -2106,7 +2106,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>storyverse</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>storyverse</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>storyverse</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>storyverse</t>
         </is>
       </c>
     </row>
@@ -7655,7 +7655,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>storyverse</t>
         </is>
       </c>
     </row>
@@ -8864,7 +8864,7 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>storyverse</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Commit the outputs of Mike's own export run
Mike re-ran 00-export.ipynb after applying EdB's corrections. The
regenerated works files reproduce, independently, exactly the values
this session had computed by applying step 9 by hand: german Other 60 /
Britain 32 / Rome 30 / France 21, french France 148 / Britain 64 /
Other 55 / Rome 46, with Willehalm von Orlens back to Other via the
automatic route and Ille et Galeron to Other via its override. That is
a genuine end-to-end check of the pipeline, not just of the data.

The linkage files show a large diff but are content-identical: 0 of
2,092 French and 0 of 1,381 German records differ once sorted, so it is
purely record ordering from the rebuild. The notebook loses one trailing
empty code cell.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/french_works.xlsx
+++ b/data/french_works.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,7 +427,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>